<commit_message>
feat(data): add fray cyclones player statistics CSV and update database and Excel output
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -15,6 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyclo Winter 2026 Game 1" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyclo Winter 2026 Game 2" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyclo Winter 2026 Game 3" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cyclo Winter 2026 Game 4" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$H$2</definedName>
@@ -24,6 +25,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Winter 2026 Game 1'!$A$1:$Q$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Winter 2026 Game 2'!$A$1:$Q$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Winter 2026 Game 3'!$A$1:$Q$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cyclo Winter 2026 Game 4'!$A$1:$Q$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -816,29 +818,29 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D2" t="n">
         <v>13</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.611</t>
+          <t>0.628</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.633</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.958</t>
+          <t>0.920</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.589</t>
+          <t>1.553</t>
         </is>
       </c>
     </row>
@@ -970,59 +972,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
         <v>7</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>2</v>
-      </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.700</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.700</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.846</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.600</t>
+          <t>1.538</t>
         </is>
       </c>
     </row>
@@ -1033,25 +1035,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -1063,29 +1065,29 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.462</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>2.154</t>
         </is>
       </c>
     </row>
@@ -1096,16 +1098,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" t="n">
         <v>6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -1129,26 +1131,26 @@
         <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.818</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.818</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1.571</t>
+          <t>1.273</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.428</t>
+          <t>2.091</t>
         </is>
       </c>
     </row>
@@ -1159,17 +1161,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" t="n">
         <v>7</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
       <c r="F5" t="n">
         <v>2</v>
       </c>
@@ -1189,29 +1191,29 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.091</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1.857</t>
+          <t>1.727</t>
         </is>
       </c>
     </row>
@@ -1222,16 +1224,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -1252,29 +1254,29 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.889</t>
+          <t>0.786</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.357</t>
         </is>
       </c>
     </row>
@@ -1285,19 +1287,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1318,26 +1320,26 @@
         <v>4</v>
       </c>
       <c r="M7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.545</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.545</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>0.858</t>
+          <t>1.181</t>
         </is>
       </c>
     </row>
@@ -1348,17 +1350,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
         <v>7</v>
       </c>
-      <c r="E8" t="n">
-        <v>5</v>
-      </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
@@ -1378,29 +1380,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.083</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2.250</t>
+          <t>1.833</t>
         </is>
       </c>
     </row>
@@ -1411,17 +1413,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
         <v>7</v>
       </c>
-      <c r="E9" t="n">
-        <v>4</v>
-      </c>
       <c r="F9" t="n">
         <v>3</v>
       </c>
@@ -1441,29 +1443,29 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.812</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.545</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -1474,10 +1476,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
@@ -1498,35 +1500,35 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
         <v>2</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>0.800</t>
         </is>
       </c>
     </row>
@@ -1726,16 +1728,16 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" t="n">
         <v>6</v>
       </c>
-      <c r="C14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" t="n">
-        <v>2</v>
-      </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -1756,29 +1758,29 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.334</t>
         </is>
       </c>
     </row>
@@ -1911,59 +1913,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
         <v>7</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>2</v>
-      </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.700</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.700</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.846</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.600</t>
+          <t>1.538</t>
         </is>
       </c>
     </row>
@@ -1974,25 +1976,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -2004,29 +2006,29 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.462</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>2.154</t>
         </is>
       </c>
     </row>
@@ -2037,16 +2039,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" t="n">
         <v>6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -2070,26 +2072,26 @@
         <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.818</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.818</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1.571</t>
+          <t>1.273</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.428</t>
+          <t>2.091</t>
         </is>
       </c>
     </row>
@@ -2100,17 +2102,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" t="n">
         <v>7</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
       <c r="F5" t="n">
         <v>2</v>
       </c>
@@ -2130,29 +2132,29 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.091</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1.857</t>
+          <t>1.727</t>
         </is>
       </c>
     </row>
@@ -2163,16 +2165,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -2193,29 +2195,29 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.889</t>
+          <t>0.786</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1.445</t>
+          <t>1.357</t>
         </is>
       </c>
     </row>
@@ -2226,19 +2228,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2259,26 +2261,26 @@
         <v>4</v>
       </c>
       <c r="M7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.545</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.545</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>0.858</t>
+          <t>1.181</t>
         </is>
       </c>
     </row>
@@ -2289,17 +2291,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
         <v>7</v>
       </c>
-      <c r="E8" t="n">
-        <v>5</v>
-      </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
@@ -2319,29 +2321,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.083</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2.250</t>
+          <t>1.833</t>
         </is>
       </c>
     </row>
@@ -2352,17 +2354,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
         <v>7</v>
       </c>
-      <c r="E9" t="n">
-        <v>4</v>
-      </c>
       <c r="F9" t="n">
         <v>3</v>
       </c>
@@ -2382,29 +2384,29 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.812</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.545</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -2415,10 +2417,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
@@ -2439,35 +2441,35 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
         <v>2</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>0.800</t>
         </is>
       </c>
     </row>
@@ -2667,16 +2669,16 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" t="n">
         <v>6</v>
       </c>
-      <c r="C14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" t="n">
-        <v>2</v>
-      </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -2697,29 +2699,29 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.334</t>
         </is>
       </c>
     </row>
@@ -2730,59 +2732,59 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>103</v>
+        <v>147</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>95</v>
+        <v>137</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>7</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>0.611</t>
+          <t>0.628</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.633</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>0.958</t>
+          <t>0.920</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>1.589</t>
+          <t>1.553</t>
         </is>
       </c>
     </row>
@@ -2915,59 +2917,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E2" t="n">
         <v>7</v>
       </c>
-      <c r="E2" t="n">
+      <c r="F2" t="n">
+        <v>2</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
         <v>5</v>
       </c>
-      <c r="F2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>2</v>
-      </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.700</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.700</t>
+          <t>0.643</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.846</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.600</t>
+          <t>1.489</t>
         </is>
       </c>
     </row>
@@ -2978,25 +2980,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
@@ -3008,29 +3010,29 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="M3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.733</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.462</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>1.600</t>
+          <t>2.195</t>
         </is>
       </c>
     </row>
@@ -3041,16 +3043,16 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C4" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
+        <v>9</v>
+      </c>
+      <c r="E4" t="n">
         <v>6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -3074,11 +3076,11 @@
         <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.818</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -3088,12 +3090,12 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1.571</t>
+          <t>1.273</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.321</t>
+          <t>2.023</t>
         </is>
       </c>
     </row>
@@ -3104,17 +3106,17 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
+        <v>11</v>
+      </c>
+      <c r="D5" t="n">
         <v>7</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>4</v>
       </c>
-      <c r="E5" t="n">
-        <v>1</v>
-      </c>
       <c r="F5" t="n">
         <v>2</v>
       </c>
@@ -3134,29 +3136,29 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="M5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.091</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>1.911</t>
+          <t>1.758</t>
         </is>
       </c>
     </row>
@@ -3167,16 +3169,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E6" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -3197,14 +3199,14 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.571</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -3214,12 +3216,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.889</t>
+          <t>0.786</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>1.489</t>
+          <t>1.386</t>
         </is>
       </c>
     </row>
@@ -3230,19 +3232,19 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -3263,26 +3265,26 @@
         <v>4</v>
       </c>
       <c r="M7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.545</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.583</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0.429</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>0.929</t>
+          <t>1.219</t>
         </is>
       </c>
     </row>
@@ -3293,17 +3295,17 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C8" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D8" t="n">
+        <v>9</v>
+      </c>
+      <c r="E8" t="n">
         <v>7</v>
       </c>
-      <c r="E8" t="n">
-        <v>5</v>
-      </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
@@ -3323,29 +3325,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.375</t>
+          <t>1.083</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2.250</t>
+          <t>1.833</t>
         </is>
       </c>
     </row>
@@ -3356,17 +3358,17 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" t="n">
         <v>7</v>
       </c>
-      <c r="E9" t="n">
-        <v>4</v>
-      </c>
       <c r="F9" t="n">
         <v>3</v>
       </c>
@@ -3386,29 +3388,29 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.812</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.545</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -3419,10 +3421,10 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D10" t="n">
         <v>2</v>
@@ -3443,35 +3445,35 @@
         <v>0</v>
       </c>
       <c r="J10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M10" t="n">
         <v>2</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.400</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>0.733</t>
         </is>
       </c>
     </row>
@@ -3671,16 +3673,16 @@
         </is>
       </c>
       <c r="B14" t="n">
+        <v>11</v>
+      </c>
+      <c r="C14" t="n">
+        <v>9</v>
+      </c>
+      <c r="D14" t="n">
         <v>6</v>
       </c>
-      <c r="C14" t="n">
-        <v>4</v>
-      </c>
-      <c r="D14" t="n">
-        <v>2</v>
-      </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F14" t="n">
         <v>0</v>
@@ -3701,29 +3703,29 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
+          <t>0.727</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
           <t>0.667</t>
         </is>
       </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>0.500</t>
-        </is>
-      </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.167</t>
+          <t>1.394</t>
         </is>
       </c>
     </row>
@@ -3734,59 +3736,59 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>103</v>
+        <v>147</v>
       </c>
       <c r="C16" s="2" t="n">
-        <v>95</v>
+        <v>137</v>
       </c>
       <c r="D16" s="2" t="n">
-        <v>58</v>
+        <v>86</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>7</v>
       </c>
       <c r="J16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L16" s="2" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="M16" s="2" t="n">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>0.611</t>
+          <t>0.628</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.633</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>0.958</t>
+          <t>0.920</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>1.589</t>
+          <t>1.553</t>
         </is>
       </c>
     </row>
@@ -6491,4 +6493,819 @@
   <autoFilter ref="A1:Q12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HRO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RBI</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OBP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SLG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>6</v>
+      </c>
+      <c r="M3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2.200</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>3.200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bryce</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" t="n">
+        <v>3</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cory</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>2</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Kap</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>2</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>4</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kunal</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n">
+        <v>4</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kyla</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>1</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>0.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Taylor</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>5</v>
+      </c>
+      <c r="C11" t="n">
+        <v>5</v>
+      </c>
+      <c r="D11" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0.800</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.800</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>0.800</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1.600</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TEAM TOTALS</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="M13" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>0.833</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q11"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
chore: Cyclones game updates 2026-03-19
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -18,6 +18,7 @@
     <sheet name="Cyclo Winter 2026 Game 4" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Cyclo Winter 2026 Game 5" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Cyclo Winter 2026 Game 6" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Cyclo Winter 2026 Game 7" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$H$2</definedName>
@@ -30,6 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Cyclo Winter 2026 Game 4'!$A$1:$Q$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Cyclo Winter 2026 Game 5'!$A$1:$Q$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Cyclo Winter 2026 Game 6'!$A$1:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Cyclo Winter 2026 Game 7'!$A$1:$Q$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2505,6 +2507,884 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HRO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RBI</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OBP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SLG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>3</v>
+      </c>
+      <c r="D2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1.667</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>2</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Bryce</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Cory</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>0.666</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>1</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Kap</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" t="n">
+        <v>3</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Kunal</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rafael</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>3</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>1</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>1.333</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1.666</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Ramos</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n">
+        <v>3</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>1</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.333</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1.333</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C11" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" t="n">
+        <v>2</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1.333</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Taylor</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" t="n">
+        <v>1</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1.250</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TEAM TOTALS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>0.559</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>0.559</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>1.029</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>1.588</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2578,29 +3458,29 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
         <v>17</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.633</t>
+          <t>0.622</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.634</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.979</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.623</t>
+          <t>1.620</t>
         </is>
       </c>
     </row>
@@ -2732,19 +3612,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -2765,26 +3645,26 @@
         <v>5</v>
       </c>
       <c r="M2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.850</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.471</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -2858,13 +3738,13 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="n">
         <v>17</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -2876,10 +3756,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -2888,29 +3768,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.733</t>
+          <t>0.706</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.733</t>
+          <t>0.706</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1.533</t>
+          <t>1.588</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.266</t>
+          <t>2.294</t>
         </is>
       </c>
     </row>
@@ -2984,19 +3864,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
         <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -3017,26 +3897,26 @@
         <v>8</v>
       </c>
       <c r="M6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.250</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.231</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -3047,16 +3927,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -3077,29 +3957,29 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.615</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.615</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -3110,59 +3990,59 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
         <v>9</v>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>8</v>
-      </c>
       <c r="M8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.810</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.471</t>
+          <t>1.477</t>
         </is>
       </c>
     </row>
@@ -3173,19 +4053,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
         <v>6</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -3203,29 +4083,29 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M9" t="n">
         <v>7</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.647</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.647</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.941</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.588</t>
         </is>
       </c>
     </row>
@@ -3236,59 +4116,59 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D10" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" t="n">
         <v>11</v>
       </c>
-      <c r="E10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" t="n">
-        <v>9</v>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.176</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.072</t>
+          <t>1.941</t>
         </is>
       </c>
     </row>
@@ -3488,13 +4368,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C14" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -3506,7 +4386,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -3518,29 +4398,29 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="M14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.556</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.556</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.778</t>
         </is>
       </c>
     </row>
@@ -3551,13 +4431,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
@@ -3566,13 +4446,13 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -3584,26 +4464,26 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.273</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.273</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.455</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.728</t>
         </is>
       </c>
     </row>
@@ -3677,59 +4557,59 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>9</v>
+      </c>
+      <c r="M17" t="n">
         <v>6</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>7</v>
-      </c>
-      <c r="M17" t="n">
-        <v>4</v>
-      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.231</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.846</t>
         </is>
       </c>
     </row>
@@ -3740,19 +4620,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -3770,29 +4650,29 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.334</t>
+          <t>1.307</t>
         </is>
       </c>
     </row>
@@ -3925,19 +4805,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -3958,26 +4838,26 @@
         <v>5</v>
       </c>
       <c r="M2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.850</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.471</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -4051,13 +4931,13 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="n">
         <v>17</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -4069,10 +4949,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -4081,29 +4961,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.733</t>
+          <t>0.706</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.733</t>
+          <t>0.706</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1.533</t>
+          <t>1.588</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.266</t>
+          <t>2.294</t>
         </is>
       </c>
     </row>
@@ -4177,19 +5057,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
         <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -4210,26 +5090,26 @@
         <v>8</v>
       </c>
       <c r="M6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.250</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.231</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -4240,16 +5120,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -4270,29 +5150,29 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.615</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.615</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.615</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -4303,59 +5183,59 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
         <v>9</v>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>8</v>
-      </c>
       <c r="M8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.810</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.471</t>
+          <t>1.477</t>
         </is>
       </c>
     </row>
@@ -4366,19 +5246,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
         <v>6</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -4396,29 +5276,29 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M9" t="n">
         <v>7</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.647</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.647</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.941</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.285</t>
+          <t>1.588</t>
         </is>
       </c>
     </row>
@@ -4429,59 +5309,59 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D10" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" t="n">
         <v>11</v>
       </c>
-      <c r="E10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" t="n">
-        <v>9</v>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.176</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.072</t>
+          <t>1.941</t>
         </is>
       </c>
     </row>
@@ -4681,13 +5561,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C14" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -4699,7 +5579,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -4711,29 +5591,29 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="M14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.556</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.556</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.778</t>
         </is>
       </c>
     </row>
@@ -4744,13 +5624,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
@@ -4759,13 +5639,13 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -4777,26 +5657,26 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.273</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.273</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.455</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.728</t>
         </is>
       </c>
     </row>
@@ -4870,59 +5750,59 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>9</v>
+      </c>
+      <c r="M17" t="n">
         <v>6</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>7</v>
-      </c>
-      <c r="M17" t="n">
-        <v>4</v>
-      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.231</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.846</t>
         </is>
       </c>
     </row>
@@ -4933,19 +5813,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -4963,29 +5843,29 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.334</t>
+          <t>1.307</t>
         </is>
       </c>
     </row>
@@ -4996,28 +5876,28 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>188</v>
+        <v>222</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>3</v>
@@ -5026,29 +5906,29 @@
         <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>0.633</t>
+          <t>0.622</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.634</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>0.979</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>1.623</t>
+          <t>1.620</t>
         </is>
       </c>
     </row>
@@ -5181,19 +6061,19 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="C2" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="D2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -5214,26 +6094,26 @@
         <v>5</v>
       </c>
       <c r="M2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.650</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.611</t>
+          <t>0.619</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.850</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.435</t>
+          <t>1.469</t>
         </is>
       </c>
     </row>
@@ -5307,13 +6187,13 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C4" t="n">
         <v>17</v>
       </c>
-      <c r="C4" t="n">
-        <v>15</v>
-      </c>
       <c r="D4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -5325,10 +6205,10 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -5337,29 +6217,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M4" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.733</t>
+          <t>0.706</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.765</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>1.533</t>
+          <t>1.588</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.298</t>
+          <t>2.338</t>
         </is>
       </c>
     </row>
@@ -5433,19 +6313,19 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
         <v>7</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
@@ -5466,26 +6346,26 @@
         <v>8</v>
       </c>
       <c r="M6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.706</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.385</t>
+          <t>1.250</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.171</t>
+          <t>1.956</t>
         </is>
       </c>
     </row>
@@ -5496,16 +6376,16 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>2</v>
@@ -5526,29 +6406,29 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="M7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.615</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.588</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.643</t>
+          <t>1.463</t>
         </is>
       </c>
     </row>
@@ -5559,59 +6439,59 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D8" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="E8" t="n">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
         <v>9</v>
       </c>
-      <c r="F8" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0</v>
-      </c>
-      <c r="K8" t="n">
-        <v>0</v>
-      </c>
-      <c r="L8" t="n">
-        <v>8</v>
-      </c>
       <c r="M8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.682</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.810</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.491</t>
+          <t>1.492</t>
         </is>
       </c>
     </row>
@@ -5622,19 +6502,19 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D9" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E9" t="n">
         <v>6</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -5652,29 +6532,29 @@
         <v>1</v>
       </c>
       <c r="L9" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="M9" t="n">
         <v>7</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.571</t>
+          <t>0.647</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.684</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.941</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>1.339</t>
+          <t>1.625</t>
         </is>
       </c>
     </row>
@@ -5685,59 +6565,59 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C10" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D10" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>7</v>
+      </c>
+      <c r="M10" t="n">
         <v>11</v>
       </c>
-      <c r="E10" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>2</v>
-      </c>
-      <c r="H10" t="n">
-        <v>1</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" t="n">
-        <v>9</v>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.176</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.072</t>
+          <t>1.941</t>
         </is>
       </c>
     </row>
@@ -5937,13 +6817,13 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C14" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" t="n">
         <v>2</v>
@@ -5955,7 +6835,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -5967,29 +6847,29 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="M14" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.556</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.556</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.778</t>
         </is>
       </c>
     </row>
@@ -6000,13 +6880,13 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
         <v>2</v>
@@ -6015,13 +6895,13 @@
         <v>0</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -6033,26 +6913,26 @@
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.273</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.400</t>
+          <t>0.429</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>0.455</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>0.650</t>
+          <t>0.884</t>
         </is>
       </c>
     </row>
@@ -6126,59 +7006,59 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C17" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E17" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" t="n">
+        <v>9</v>
+      </c>
+      <c r="M17" t="n">
         <v>6</v>
       </c>
-      <c r="E17" t="n">
-        <v>2</v>
-      </c>
-      <c r="F17" t="n">
-        <v>3</v>
-      </c>
-      <c r="G17" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" t="n">
-        <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0</v>
-      </c>
-      <c r="K17" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" t="n">
-        <v>7</v>
-      </c>
-      <c r="M17" t="n">
-        <v>4</v>
-      </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>0.615</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.231</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1.800</t>
+          <t>1.846</t>
         </is>
       </c>
     </row>
@@ -6189,19 +7069,19 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C18" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D18" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G18" t="n">
         <v>0</v>
@@ -6219,29 +7099,29 @@
         <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="M18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
+          <t>0.615</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
           <t>0.667</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>0.727</t>
-        </is>
-      </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1.394</t>
+          <t>1.359</t>
         </is>
       </c>
     </row>
@@ -6252,28 +7132,28 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="C20" s="2" t="n">
-        <v>188</v>
+        <v>222</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>119</v>
+        <v>138</v>
       </c>
       <c r="E20" s="2" t="n">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>3</v>
@@ -6282,29 +7162,29 @@
         <v>1</v>
       </c>
       <c r="L20" s="2" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="M20" s="2" t="n">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>0.633</t>
+          <t>0.622</t>
         </is>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.634</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>0.979</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>1.623</t>
+          <t>1.620</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Cyclones game updates 2026-04-30
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -23,6 +23,7 @@
     <sheet name="Cyclo Spring 2026 Game 1" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Cyclo Spring 2026 Game 2" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Cyclo Spring 2026 Game 3" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Cyclo Spring 2026 Game 5" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$H$3</definedName>
@@ -40,6 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cyclo Spring 2026 Game 1'!$A$1:$Q$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Cyclo Spring 2026 Game 2'!$A$1:$Q$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Cyclo Spring 2026 Game 3'!$A$1:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Cyclo Spring 2026 Game 5'!$A$1:$Q$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3516,25 +3518,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -3546,29 +3548,29 @@
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1.250</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.875</t>
+          <t>2.250</t>
         </is>
       </c>
     </row>
@@ -3642,22 +3644,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
@@ -3672,29 +3674,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>3.167</t>
+          <t>2.091</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4.167</t>
+          <t>2.818</t>
         </is>
       </c>
     </row>
@@ -3705,16 +3707,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -3735,10 +3737,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -3752,12 +3754,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -3831,22 +3833,22 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D7" t="n">
         <v>9</v>
       </c>
-      <c r="C7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -3861,29 +3863,29 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1.111</t>
+          <t>1.231</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.667</t>
+          <t>1.923</t>
         </is>
       </c>
     </row>
@@ -3957,16 +3959,16 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" t="n">
         <v>7</v>
       </c>
-      <c r="C9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -3990,26 +3992,26 @@
         <v>9</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2.429</t>
+          <t>1.727</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>3.143</t>
+          <t>2.363</t>
         </is>
       </c>
     </row>
@@ -4020,59 +4022,59 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D10" t="n">
         <v>11</v>
       </c>
-      <c r="C10" t="n">
+      <c r="E10" t="n">
         <v>11</v>
       </c>
-      <c r="D10" t="n">
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" t="n">
         <v>6</v>
       </c>
-      <c r="E10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>4</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3</v>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.090</t>
+          <t>1.376</t>
         </is>
       </c>
     </row>
@@ -4083,16 +4085,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -4104,7 +4106,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -4113,19 +4115,19 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4135,7 +4137,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.292</t>
         </is>
       </c>
     </row>
@@ -4146,59 +4148,59 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
         <v>8</v>
       </c>
-      <c r="C12" t="n">
+      <c r="M12" t="n">
         <v>7</v>
       </c>
-      <c r="D12" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M12" t="n">
-        <v>5</v>
-      </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.909</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.750</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>1.636</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2.179</t>
+          <t>2.469</t>
         </is>
       </c>
     </row>
@@ -4272,25 +4274,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" t="n">
         <v>6</v>
       </c>
-      <c r="E14" t="n">
-        <v>5</v>
-      </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -4302,29 +4304,29 @@
         <v>2</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.181</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -4335,19 +4337,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -4365,29 +4367,29 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -4398,16 +4400,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -4416,7 +4418,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -4425,32 +4427,32 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.444</t>
+          <t>0.462</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>0.444</t>
+          <t>0.462</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0.444</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>0.888</t>
+          <t>1.154</t>
         </is>
       </c>
     </row>
@@ -4461,59 +4463,59 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="D18" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="C18" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>64</v>
-      </c>
       <c r="E18" s="2" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>0.653</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>0.646</t>
+          <t>0.687</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>1.214</t>
+          <t>1.208</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>1.860</t>
+          <t>1.895</t>
         </is>
       </c>
     </row>
@@ -7220,6 +7222,884 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HRO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RBI</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OBP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SLG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0.400</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.400</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.800</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Baxter</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bryce</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cory</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Erin</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kap</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kyla</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1.400</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1.250</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TEAM TOTALS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>0.761</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>0.761</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>1.196</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>1.957</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7293,29 +8173,29 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
         <v>21</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.638</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>1.074</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.729</t>
         </is>
       </c>
     </row>
@@ -7331,29 +8211,29 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
         <v>21</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.638</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>1.074</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.729</t>
         </is>
       </c>
     </row>
@@ -7485,59 +8365,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
         <v>11</v>
       </c>
-      <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>7</v>
-      </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>1.094</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.607</t>
+          <t>1.782</t>
         </is>
       </c>
     </row>
@@ -7611,22 +8491,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>6</v>
@@ -7641,29 +8521,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.786</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.783</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -7737,16 +8617,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -7767,10 +8647,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -7784,12 +8664,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -7863,22 +8743,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -7893,29 +8773,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.241</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.880</t>
+          <t>1.965</t>
         </is>
       </c>
     </row>
@@ -7989,16 +8869,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -8022,26 +8902,26 @@
         <v>19</v>
       </c>
       <c r="M10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.348</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.957</t>
+          <t>1.815</t>
         </is>
       </c>
     </row>
@@ -8052,16 +8932,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C11" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -8082,29 +8962,29 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
+        <v>14</v>
+      </c>
+      <c r="M11" t="n">
         <v>13</v>
       </c>
-      <c r="M11" t="n">
-        <v>10</v>
-      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0.719</t>
+          <t>0.757</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.344</t>
+          <t>1.433</t>
         </is>
       </c>
     </row>
@@ -8115,16 +8995,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -8136,7 +9016,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -8145,19 +9025,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -8167,7 +9047,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.167</t>
         </is>
       </c>
     </row>
@@ -8178,59 +9058,59 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
         <v>17</v>
       </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="n">
-        <v>13</v>
-      </c>
       <c r="M13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>1.083</t>
+          <t>1.214</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.791</t>
+          <t>1.964</t>
         </is>
       </c>
     </row>
@@ -8304,25 +9184,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -8334,10 +9214,10 @@
         <v>2</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -8351,12 +9231,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.829</t>
+          <t>0.900</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -8430,19 +9310,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -8460,29 +9340,29 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M17" t="n">
         <v>5</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.910</t>
+          <t>1.133</t>
         </is>
       </c>
     </row>
@@ -8682,16 +9562,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>3</v>
@@ -8700,7 +9580,7 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -8709,32 +9589,32 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.962</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.454</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -8930,59 +9810,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
         <v>11</v>
       </c>
-      <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>7</v>
-      </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>1.094</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.607</t>
+          <t>1.782</t>
         </is>
       </c>
     </row>
@@ -9056,22 +9936,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>6</v>
@@ -9086,29 +9966,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.786</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.783</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -9182,16 +10062,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -9212,10 +10092,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -9229,12 +10109,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -9308,22 +10188,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -9338,29 +10218,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.241</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.880</t>
+          <t>1.965</t>
         </is>
       </c>
     </row>
@@ -9434,16 +10314,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -9467,26 +10347,26 @@
         <v>19</v>
       </c>
       <c r="M10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.348</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.957</t>
+          <t>1.815</t>
         </is>
       </c>
     </row>
@@ -9497,16 +10377,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C11" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -9527,29 +10407,29 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
+        <v>14</v>
+      </c>
+      <c r="M11" t="n">
         <v>13</v>
       </c>
-      <c r="M11" t="n">
-        <v>10</v>
-      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0.719</t>
+          <t>0.757</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.344</t>
+          <t>1.433</t>
         </is>
       </c>
     </row>
@@ -9560,16 +10440,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -9581,7 +10461,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -9590,19 +10470,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -9612,7 +10492,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.167</t>
         </is>
       </c>
     </row>
@@ -9623,59 +10503,59 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
         <v>17</v>
       </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="n">
-        <v>13</v>
-      </c>
       <c r="M13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>1.083</t>
+          <t>1.214</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.791</t>
+          <t>1.964</t>
         </is>
       </c>
     </row>
@@ -9749,25 +10629,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -9779,10 +10659,10 @@
         <v>2</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -9796,12 +10676,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.829</t>
+          <t>0.900</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -9875,19 +10755,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -9905,29 +10785,29 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M17" t="n">
         <v>5</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.910</t>
+          <t>1.133</t>
         </is>
       </c>
     </row>
@@ -10127,16 +11007,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>3</v>
@@ -10145,7 +11025,7 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -10154,32 +11034,32 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.962</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.454</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -10253,59 +11133,59 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>337</v>
+        <v>385</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>320</v>
+        <v>366</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>4</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>0.638</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>1.074</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.729</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: Cyclones game updates 2026-04-30 (#5)
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -23,6 +23,7 @@
     <sheet name="Cyclo Spring 2026 Game 1" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Cyclo Spring 2026 Game 2" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Cyclo Spring 2026 Game 3" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Cyclo Spring 2026 Game 5" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$H$3</definedName>
@@ -40,6 +41,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Cyclo Spring 2026 Game 1'!$A$1:$Q$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Cyclo Spring 2026 Game 2'!$A$1:$Q$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Cyclo Spring 2026 Game 3'!$A$1:$Q$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Cyclo Spring 2026 Game 5'!$A$1:$Q$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3516,25 +3518,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I2" t="n">
         <v>0</v>
@@ -3546,29 +3548,29 @@
         <v>1</v>
       </c>
       <c r="L2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="M2" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>1.250</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.875</t>
+          <t>2.250</t>
         </is>
       </c>
     </row>
@@ -3642,22 +3644,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>4</v>
@@ -3672,29 +3674,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.727</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>3.167</t>
+          <t>2.091</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4.167</t>
+          <t>2.818</t>
         </is>
       </c>
     </row>
@@ -3705,16 +3707,16 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -3735,10 +3737,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M5" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -3752,12 +3754,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -3831,22 +3833,22 @@
         </is>
       </c>
       <c r="B7" t="n">
+        <v>13</v>
+      </c>
+      <c r="C7" t="n">
+        <v>13</v>
+      </c>
+      <c r="D7" t="n">
         <v>9</v>
       </c>
-      <c r="C7" t="n">
-        <v>9</v>
-      </c>
-      <c r="D7" t="n">
-        <v>5</v>
-      </c>
       <c r="E7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="n">
         <v>1</v>
@@ -3861,29 +3863,29 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>0.556</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>1.111</t>
+          <t>1.231</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>1.667</t>
+          <t>1.923</t>
         </is>
       </c>
     </row>
@@ -3957,16 +3959,16 @@
         </is>
       </c>
       <c r="B9" t="n">
+        <v>11</v>
+      </c>
+      <c r="C9" t="n">
+        <v>11</v>
+      </c>
+      <c r="D9" t="n">
         <v>7</v>
       </c>
-      <c r="C9" t="n">
-        <v>7</v>
-      </c>
-      <c r="D9" t="n">
-        <v>5</v>
-      </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
         <v>0</v>
@@ -3990,26 +3992,26 @@
         <v>9</v>
       </c>
       <c r="M9" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>0.714</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2.429</t>
+          <t>1.727</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>3.143</t>
+          <t>2.363</t>
         </is>
       </c>
     </row>
@@ -4020,59 +4022,59 @@
         </is>
       </c>
       <c r="B10" t="n">
+        <v>16</v>
+      </c>
+      <c r="C10" t="n">
+        <v>16</v>
+      </c>
+      <c r="D10" t="n">
         <v>11</v>
       </c>
-      <c r="C10" t="n">
+      <c r="E10" t="n">
         <v>11</v>
       </c>
-      <c r="D10" t="n">
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>5</v>
+      </c>
+      <c r="M10" t="n">
         <v>6</v>
       </c>
-      <c r="E10" t="n">
-        <v>6</v>
-      </c>
-      <c r="F10" t="n">
-        <v>0</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" t="n">
-        <v>0</v>
-      </c>
-      <c r="L10" t="n">
-        <v>4</v>
-      </c>
-      <c r="M10" t="n">
-        <v>3</v>
-      </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.090</t>
+          <t>1.376</t>
         </is>
       </c>
     </row>
@@ -4083,16 +4085,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -4104,7 +4106,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -4113,19 +4115,19 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M11" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.625</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -4135,7 +4137,7 @@
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.292</t>
         </is>
       </c>
     </row>
@@ -4146,59 +4148,59 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>12</v>
+      </c>
+      <c r="C12" t="n">
+        <v>11</v>
+      </c>
+      <c r="D12" t="n">
+        <v>10</v>
+      </c>
+      <c r="E12" t="n">
+        <v>6</v>
+      </c>
+      <c r="F12" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
         <v>8</v>
       </c>
-      <c r="C12" t="n">
+      <c r="M12" t="n">
         <v>7</v>
       </c>
-      <c r="D12" t="n">
-        <v>6</v>
-      </c>
-      <c r="E12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M12" t="n">
-        <v>5</v>
-      </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.909</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.750</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>1.636</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2.179</t>
+          <t>2.469</t>
         </is>
       </c>
     </row>
@@ -4272,25 +4274,25 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D14" t="n">
+        <v>9</v>
+      </c>
+      <c r="E14" t="n">
         <v>6</v>
       </c>
-      <c r="E14" t="n">
-        <v>5</v>
-      </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -4302,29 +4304,29 @@
         <v>2</v>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="M14" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.562</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.636</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>1.181</t>
+          <t>1.437</t>
         </is>
       </c>
     </row>
@@ -4335,19 +4337,19 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -4365,29 +4367,29 @@
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>0.833</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -4398,16 +4400,16 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C16" t="n">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D16" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E16" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F16" t="n">
         <v>0</v>
@@ -4416,7 +4418,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
         <v>0</v>
@@ -4425,32 +4427,32 @@
         <v>0</v>
       </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M16" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>0.444</t>
+          <t>0.462</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>0.444</t>
+          <t>0.462</t>
         </is>
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0.444</t>
+          <t>0.692</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>0.888</t>
+          <t>1.154</t>
         </is>
       </c>
     </row>
@@ -4461,59 +4463,59 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
+        <v>147</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>144</v>
+      </c>
+      <c r="D18" s="2" t="n">
         <v>99</v>
       </c>
-      <c r="C18" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="D18" s="2" t="n">
-        <v>64</v>
-      </c>
       <c r="E18" s="2" t="n">
-        <v>40</v>
+        <v>65</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="M18" s="2" t="n">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>0.653</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>0.646</t>
+          <t>0.687</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>1.214</t>
+          <t>1.208</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>1.860</t>
+          <t>1.895</t>
         </is>
       </c>
     </row>
@@ -7220,6 +7222,884 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FFFFFF00"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>PA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>AB</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>1B</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>2B</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>3B</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>HR</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SF</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>HRO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>RBI</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OBP</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SLG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>OPS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Alex</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n">
+        <v>4</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Anthony</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>2</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0.400</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.400</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.800</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1.200</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Baxter</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E4" t="n">
+        <v>4</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
+        <v>4</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Bryce</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>2</v>
+      </c>
+      <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>1.500</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2.500</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Cory</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Devon</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" t="n">
+        <v>5</v>
+      </c>
+      <c r="D7" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" t="n">
+        <v>5</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" t="n">
+        <v>3</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Erin</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" t="n">
+        <v>3</v>
+      </c>
+      <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>2</v>
+      </c>
+      <c r="M8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>0.667</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1.334</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Kap</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n">
+        <v>4</v>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>2</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" t="n">
+        <v>2</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>3.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Kyla</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" t="n">
+        <v>5</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>2</v>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.600</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>1.400</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2.000</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Paul</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n">
+        <v>4</v>
+      </c>
+      <c r="D11" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.750</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>1.000</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Stephen</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n">
+        <v>4</v>
+      </c>
+      <c r="D12" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1</v>
+      </c>
+      <c r="M12" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.500</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>1.250</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1.750</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TEAM TOTALS</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="M14" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>0.761</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>0.761</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>1.196</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>1.957</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Q12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -7293,29 +8173,29 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="n">
         <v>21</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>0.638</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>1.074</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.729</t>
         </is>
       </c>
     </row>
@@ -7331,29 +8211,29 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="n">
         <v>21</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>0.638</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>1.074</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.729</t>
         </is>
       </c>
     </row>
@@ -7485,59 +8365,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
         <v>11</v>
       </c>
-      <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>7</v>
-      </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>1.094</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.607</t>
+          <t>1.782</t>
         </is>
       </c>
     </row>
@@ -7611,22 +8491,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>6</v>
@@ -7641,29 +8521,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.786</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.783</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -7737,16 +8617,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -7767,10 +8647,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -7784,12 +8664,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -7863,22 +8743,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -7893,29 +8773,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.241</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.880</t>
+          <t>1.965</t>
         </is>
       </c>
     </row>
@@ -7989,16 +8869,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -8022,26 +8902,26 @@
         <v>19</v>
       </c>
       <c r="M10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.348</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.957</t>
+          <t>1.815</t>
         </is>
       </c>
     </row>
@@ -8052,16 +8932,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C11" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -8082,29 +8962,29 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
+        <v>14</v>
+      </c>
+      <c r="M11" t="n">
         <v>13</v>
       </c>
-      <c r="M11" t="n">
-        <v>10</v>
-      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0.719</t>
+          <t>0.757</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.344</t>
+          <t>1.433</t>
         </is>
       </c>
     </row>
@@ -8115,16 +8995,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -8136,7 +9016,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -8145,19 +9025,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -8167,7 +9047,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.167</t>
         </is>
       </c>
     </row>
@@ -8178,59 +9058,59 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
         <v>17</v>
       </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="n">
-        <v>13</v>
-      </c>
       <c r="M13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>1.083</t>
+          <t>1.214</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.791</t>
+          <t>1.964</t>
         </is>
       </c>
     </row>
@@ -8304,25 +9184,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -8334,10 +9214,10 @@
         <v>2</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -8351,12 +9231,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.829</t>
+          <t>0.900</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -8430,19 +9310,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -8460,29 +9340,29 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M17" t="n">
         <v>5</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.910</t>
+          <t>1.133</t>
         </is>
       </c>
     </row>
@@ -8682,16 +9562,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>3</v>
@@ -8700,7 +9580,7 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -8709,32 +9589,32 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.962</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.454</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -8930,59 +9810,59 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C2" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="D2" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F2" t="n">
+        <v>7</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L2" t="n">
         <v>11</v>
       </c>
-      <c r="F2" t="n">
-        <v>6</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="n">
-        <v>1</v>
-      </c>
-      <c r="L2" t="n">
-        <v>7</v>
-      </c>
       <c r="M2" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>0.643</t>
+          <t>0.688</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>1.094</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>1.607</t>
+          <t>1.782</t>
         </is>
       </c>
     </row>
@@ -9056,22 +9936,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F4" t="n">
         <v>10</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
         <v>6</v>
@@ -9086,29 +9966,29 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="M4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>0.783</t>
+          <t>0.714</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2.000</t>
+          <t>1.786</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2.783</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -9182,16 +10062,16 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="C6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F6" t="n">
         <v>1</v>
@@ -9212,10 +10092,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="M6" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -9229,12 +10109,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>1.750</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2.750</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -9308,22 +10188,22 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="D8" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F8" t="n">
         <v>3</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" t="n">
         <v>2</v>
@@ -9338,29 +10218,29 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M8" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>0.680</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.241</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>1.880</t>
+          <t>1.965</t>
         </is>
       </c>
     </row>
@@ -9434,16 +10314,16 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F10" t="n">
         <v>2</v>
@@ -9467,26 +10347,26 @@
         <v>19</v>
       </c>
       <c r="M10" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.348</t>
+          <t>1.222</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>1.957</t>
+          <t>1.815</t>
         </is>
       </c>
     </row>
@@ -9497,16 +10377,16 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C11" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="D11" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E11" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F11" t="n">
         <v>1</v>
@@ -9527,29 +10407,29 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
+        <v>14</v>
+      </c>
+      <c r="M11" t="n">
         <v>13</v>
       </c>
-      <c r="M11" t="n">
-        <v>10</v>
-      </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0.719</t>
+          <t>0.757</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>1.344</t>
+          <t>1.433</t>
         </is>
       </c>
     </row>
@@ -9560,16 +10440,16 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F12" t="n">
         <v>1</v>
@@ -9581,7 +10461,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J12" t="n">
         <v>0</v>
@@ -9590,19 +10470,19 @@
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="M12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.500</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -9612,7 +10492,7 @@
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>1.167</t>
         </is>
       </c>
     </row>
@@ -9623,59 +10503,59 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C13" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="D13" t="n">
+        <v>21</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" t="n">
         <v>17</v>
       </c>
-      <c r="E13" t="n">
-        <v>10</v>
-      </c>
-      <c r="F13" t="n">
-        <v>6</v>
-      </c>
-      <c r="G13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>1</v>
-      </c>
-      <c r="L13" t="n">
-        <v>13</v>
-      </c>
       <c r="M13" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.750</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>1.083</t>
+          <t>1.214</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>1.791</t>
+          <t>1.964</t>
         </is>
       </c>
     </row>
@@ -9749,25 +10629,25 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C15" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="D15" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E15" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F15" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
@@ -9779,10 +10659,10 @@
         <v>2</v>
       </c>
       <c r="L15" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="M15" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -9796,12 +10676,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.829</t>
+          <t>0.900</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.429</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -9875,19 +10755,19 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="C17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="D17" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -9905,29 +10785,29 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M17" t="n">
         <v>5</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.455</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>0.910</t>
+          <t>1.133</t>
         </is>
       </c>
     </row>
@@ -10127,16 +11007,16 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C21" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="D21" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="E21" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F21" t="n">
         <v>3</v>
@@ -10145,7 +11025,7 @@
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
@@ -10154,32 +11034,32 @@
         <v>0</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M21" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>0.545</t>
+          <t>0.538</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.962</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1.454</t>
+          <t>1.500</t>
         </is>
       </c>
     </row>
@@ -10253,59 +11133,59 @@
         </is>
       </c>
       <c r="B24" s="2" t="n">
-        <v>337</v>
+        <v>385</v>
       </c>
       <c r="C24" s="2" t="n">
-        <v>320</v>
+        <v>366</v>
       </c>
       <c r="D24" s="2" t="n">
-        <v>202</v>
+        <v>237</v>
       </c>
       <c r="E24" s="2" t="n">
-        <v>123</v>
+        <v>148</v>
       </c>
       <c r="F24" s="2" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="G24" s="2" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>4</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L24" s="2" t="n">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="M24" s="2" t="n">
-        <v>156</v>
+        <v>180</v>
       </c>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>0.631</t>
+          <t>0.648</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>0.638</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>1.074</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.729</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correct player statistics for Stephen and Kap in game data
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -10167,12 +10167,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.997</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.619</t>
+          <t>1.618</t>
         </is>
       </c>
     </row>
@@ -20479,10 +20479,10 @@
         <v>39</v>
       </c>
       <c r="E15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
@@ -20517,12 +20517,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>1.170</t>
+          <t>1.151</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.916</t>
+          <t>1.897</t>
         </is>
       </c>
     </row>
@@ -25688,10 +25688,10 @@
         <v>39</v>
       </c>
       <c r="E15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
@@ -25726,12 +25726,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>1.170</t>
+          <t>1.151</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.916</t>
+          <t>1.897</t>
         </is>
       </c>
     </row>
@@ -26507,10 +26507,10 @@
         <v>486</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>24</v>
@@ -26545,12 +26545,12 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>0.997</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>1.619</t>
+          <t>1.618</t>
         </is>
       </c>
     </row>
@@ -27259,10 +27259,10 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -27297,12 +27297,12 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -27637,10 +27637,10 @@
         <v>42</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>2</v>
@@ -27675,12 +27675,12 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>1.188</t>
+          <t>1.172</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>1.830</t>
+          <t>1.814</t>
         </is>
       </c>
     </row>
@@ -29078,10 +29078,10 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -29116,12 +29116,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -29330,10 +29330,10 @@
         <v>16</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>1</v>
@@ -29368,12 +29368,12 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>1.034</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>1.586</t>
+          <t>1.552</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: correct player statistics for Stephen and Kap in game data (#18)
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -10167,12 +10167,12 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>0.997</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.619</t>
+          <t>1.618</t>
         </is>
       </c>
     </row>
@@ -20479,10 +20479,10 @@
         <v>39</v>
       </c>
       <c r="E15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
@@ -20517,12 +20517,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>1.170</t>
+          <t>1.151</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.916</t>
+          <t>1.897</t>
         </is>
       </c>
     </row>
@@ -25688,10 +25688,10 @@
         <v>39</v>
       </c>
       <c r="E15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F15" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
@@ -25726,12 +25726,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>1.170</t>
+          <t>1.151</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>1.916</t>
+          <t>1.897</t>
         </is>
       </c>
     </row>
@@ -26507,10 +26507,10 @@
         <v>486</v>
       </c>
       <c r="E29" s="2" t="n">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>24</v>
@@ -26545,12 +26545,12 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>0.997</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
         <is>
-          <t>1.619</t>
+          <t>1.618</t>
         </is>
       </c>
     </row>
@@ -27259,10 +27259,10 @@
         <v>2</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
         <v>0</v>
@@ -27297,12 +27297,12 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -27637,10 +27637,10 @@
         <v>42</v>
       </c>
       <c r="E18" s="2" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>2</v>
@@ -27675,12 +27675,12 @@
       </c>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>1.188</t>
+          <t>1.172</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>1.830</t>
+          <t>1.814</t>
         </is>
       </c>
     </row>
@@ -29078,10 +29078,10 @@
         <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
         <v>0</v>
@@ -29116,12 +29116,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>1.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>2.000</t>
         </is>
       </c>
     </row>
@@ -29330,10 +29330,10 @@
         <v>16</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>1</v>
@@ -29368,12 +29368,12 @@
       </c>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>1.034</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>1.586</t>
+          <t>1.552</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: 2026 LSU game 2 player name
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -45,7 +45,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Player Summary'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cyclo Total'!$A$1:$Q$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cyclo Late Summer 2026 Total'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cyclo Late Summer 2026 Total'!$A$1:$Q$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Late Summer 2026 Game 1'!$A$1:$Q$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Late Summer 2026 Game 2'!$A$1:$Q$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Summer 2026 Total'!$A$1:$Q$18</definedName>
@@ -20722,16 +20722,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D19" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" t="n">
         <v>10</v>
@@ -20746,35 +20746,35 @@
         <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M19" t="n">
         <v>36</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.602</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.867</t>
+          <t>0.849</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.476</t>
+          <t>1.442</t>
         </is>
       </c>
     </row>
@@ -20785,16 +20785,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -20809,35 +20809,35 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.800</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.300</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -25931,16 +25931,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D19" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" t="n">
         <v>10</v>
@@ -25955,35 +25955,35 @@
         <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M19" t="n">
         <v>36</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.602</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.867</t>
+          <t>0.849</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.476</t>
+          <t>1.442</t>
         </is>
       </c>
     </row>
@@ -25994,16 +25994,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -26018,35 +26018,35 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.800</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.300</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -26567,7 +26567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27313,82 +27313,82 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" t="n">
         <v>6</v>
       </c>
-      <c r="C12" t="n">
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
         <v>6</v>
       </c>
-      <c r="D12" t="n">
-        <v>5</v>
-      </c>
-      <c r="E12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>4</v>
-      </c>
       <c r="M12" t="n">
         <v>2</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.778</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.378</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kyle</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -27400,7 +27400,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -27409,55 +27409,55 @@
         <v>2</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.333</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>0.583</t>
+          <t>2.333</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Rafael</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -27469,10 +27469,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -27486,32 +27486,32 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1.333</t>
+          <t>2.500</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2.333</t>
+          <t>3.500</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Rafael</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -27535,157 +27535,94 @@
         <v>3</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>1.200</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>3.500</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Stephen</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3</v>
-      </c>
-      <c r="M16" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0.600</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0.600</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>1.200</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
           <t>1.800</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>TEAM TOTALS</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D17" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E17" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F17" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="2" t="n">
+      <c r="G17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2" t="n">
+      <c r="I17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>0.656</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>0.642</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>1.172</t>
         </is>
       </c>
-      <c r="Q18" s="2" t="inlineStr">
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>1.814</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:Q15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29128,7 +29065,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kyle</t>
+          <t>Kyla</t>
         </is>
       </c>
       <c r="B11" t="n">

</xml_diff>

<commit_message>
fix: 2026 LSU game 2 player name (#19)
</commit_message>
<xml_diff>
--- a/data/output/stats.xlsx
+++ b/data/output/stats.xlsx
@@ -45,7 +45,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'League Summary'!$A$1:$H$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Player Summary'!$A$1:$Q$27</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cyclo Total'!$A$1:$Q$27</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cyclo Late Summer 2026 Total'!$A$1:$Q$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Cyclo Late Summer 2026 Total'!$A$1:$Q$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Cyclo Late Summer 2026 Game 1'!$A$1:$Q$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cyclo Late Summer 2026 Game 2'!$A$1:$Q$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Cyclo Summer 2026 Total'!$A$1:$Q$18</definedName>
@@ -20722,16 +20722,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D19" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" t="n">
         <v>10</v>
@@ -20746,35 +20746,35 @@
         <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M19" t="n">
         <v>36</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.602</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.867</t>
+          <t>0.849</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.476</t>
+          <t>1.442</t>
         </is>
       </c>
     </row>
@@ -20785,16 +20785,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -20809,35 +20809,35 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.800</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.300</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -25931,16 +25931,16 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C19" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D19" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E19" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="F19" t="n">
         <v>10</v>
@@ -25955,35 +25955,35 @@
         <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K19" t="n">
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="M19" t="n">
         <v>36</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.602</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.609</t>
+          <t>0.593</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.867</t>
+          <t>0.849</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1.476</t>
+          <t>1.442</t>
         </is>
       </c>
     </row>
@@ -25994,16 +25994,16 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C20" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E20" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" t="n">
         <v>1</v>
@@ -26018,35 +26018,35 @@
         <v>0</v>
       </c>
       <c r="J20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M20" t="n">
         <v>1</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>0.600</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>0.500</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.800</t>
+          <t>1.500</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1.300</t>
+          <t>2.500</t>
         </is>
       </c>
     </row>
@@ -26567,7 +26567,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -27313,82 +27313,82 @@
         </is>
       </c>
       <c r="B12" t="n">
+        <v>10</v>
+      </c>
+      <c r="C12" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" t="n">
         <v>6</v>
       </c>
-      <c r="C12" t="n">
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
         <v>6</v>
       </c>
-      <c r="D12" t="n">
-        <v>5</v>
-      </c>
-      <c r="E12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-      <c r="K12" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" t="n">
-        <v>4</v>
-      </c>
       <c r="M12" t="n">
         <v>2</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.667</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>0.833</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.778</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>1.833</t>
+          <t>1.378</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kyle</t>
+          <t>Paul</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n">
         <v>3</v>
       </c>
       <c r="D13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G13" t="n">
         <v>0</v>
@@ -27400,7 +27400,7 @@
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -27409,55 +27409,55 @@
         <v>2</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>0.250</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>1.333</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>0.583</t>
+          <t>2.333</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Paul</t>
+          <t>Rafael</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G14" t="n">
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
@@ -27469,10 +27469,10 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -27486,32 +27486,32 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>1.333</t>
+          <t>2.500</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
         <is>
-          <t>2.333</t>
+          <t>3.500</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Rafael</t>
+          <t>Stephen</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F15" t="n">
         <v>0</v>
@@ -27535,157 +27535,94 @@
         <v>3</v>
       </c>
       <c r="M15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.600</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2.500</t>
+          <t>1.200</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
         <is>
-          <t>3.500</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Stephen</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>5</v>
-      </c>
-      <c r="C16" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" t="n">
-        <v>2</v>
-      </c>
-      <c r="F16" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>1</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" t="n">
-        <v>3</v>
-      </c>
-      <c r="M16" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0.600</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0.600</t>
-        </is>
-      </c>
-      <c r="P16" t="inlineStr">
-        <is>
-          <t>1.200</t>
-        </is>
-      </c>
-      <c r="Q16" t="inlineStr">
-        <is>
           <t>1.800</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>TEAM TOTALS</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="C18" s="2" t="n">
+      <c r="C17" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D17" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E17" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="F18" s="2" t="n">
+      <c r="F17" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="G18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="2" t="n">
+      <c r="G17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="I18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="K18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="2" t="n">
+      <c r="I17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="M18" s="2" t="n">
+      <c r="M17" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>0.656</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>0.642</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>1.172</t>
         </is>
       </c>
-      <c r="Q18" s="2" t="inlineStr">
+      <c r="Q17" s="2" t="inlineStr">
         <is>
           <t>1.814</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q16"/>
+  <autoFilter ref="A1:Q15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -29128,7 +29065,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Kyle</t>
+          <t>Kyla</t>
         </is>
       </c>
       <c r="B11" t="n">

</xml_diff>